<commit_message>
update Peru CPUE to include tech creep; correct growth parameters to FL
</commit_message>
<xml_diff>
--- a/assessment/data/SC10_2022assessmentInputData.xlsx
+++ b/assessment/data/SC10_2022assessmentInputData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10814"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leeqi/Library/CloudStorage/GoogleDrive-leeqi@uw.edu/My Drive/SPRFMO/jjm/assessment/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://southpacificrfmo.sharepoint.com/sites/SPRFMOSCJackMackerelWorkingGroup/Shared Documents/Data repository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14BB2B41-70C3-1343-A509-2EB0A20DD8A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2BB3040E-2287-40B5-ABC1-96FD71463E9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" activeTab="4" xr2:uid="{11C67D07-EBA6-4D97-A3E6-A5FACAECFD42}"/>
+    <workbookView xWindow="840" yWindow="-120" windowWidth="28080" windowHeight="16440" activeTab="3" xr2:uid="{11C67D07-EBA6-4D97-A3E6-A5FACAECFD42}"/>
   </bookViews>
   <sheets>
     <sheet name="ageComps" sheetId="1" r:id="rId1"/>
@@ -423,9 +423,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCC02C38-8F7E-48D4-BE42-B6D35726D79C}">
   <dimension ref="A1:F27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -445,7 +445,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2021</v>
       </c>
@@ -459,7 +459,7 @@
         <v>670.16183246731998</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2021</v>
       </c>
@@ -476,7 +476,7 @@
         <v>13279.648895886301</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2021</v>
       </c>
@@ -493,7 +493,7 @@
         <v>44760.811535680899</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -510,7 +510,7 @@
         <v>107827.383916946</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2021</v>
       </c>
@@ -527,7 +527,7 @@
         <v>28181.237063751298</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2021</v>
       </c>
@@ -544,7 +544,7 @@
         <v>15482.537721409301</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2021</v>
       </c>
@@ -561,7 +561,7 @@
         <v>4128.7939220620001</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2021</v>
       </c>
@@ -578,7 +578,7 @@
         <v>427.17024803910601</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2021</v>
       </c>
@@ -595,7 +595,7 @@
         <v>110.74670539676799</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2021</v>
       </c>
@@ -612,7 +612,7 @@
         <v>221.93965880599998</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2021</v>
       </c>
@@ -629,7 +629,7 @@
         <v>10.7458646434357</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2021</v>
       </c>
@@ -646,7 +646,7 @@
         <v>4.1277274962150202E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2021</v>
       </c>
@@ -663,7 +663,7 @@
         <v>3.48499840965275</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2022</v>
       </c>
@@ -680,7 +680,7 @@
         <v>566.99602958347407</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2022</v>
       </c>
@@ -697,7 +697,7 @@
         <v>32809.856850873999</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2022</v>
       </c>
@@ -714,7 +714,7 @@
         <v>178240.213244949</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2022</v>
       </c>
@@ -731,7 +731,7 @@
         <v>7845.8419073151599</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2022</v>
       </c>
@@ -748,7 +748,7 @@
         <v>3835.6966651638604</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2022</v>
       </c>
@@ -765,7 +765,7 @@
         <v>2051.2549168066002</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2022</v>
       </c>
@@ -782,7 +782,7 @@
         <v>929.75059235101901</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2022</v>
       </c>
@@ -799,7 +799,7 @@
         <v>441.63141196245601</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2022</v>
       </c>
@@ -816,7 +816,7 @@
         <v>263.18018713831498</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2022</v>
       </c>
@@ -833,7 +833,7 @@
         <v>132.02478459123498</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2022</v>
       </c>
@@ -850,7 +850,7 @@
         <v>78.603420554523197</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2022</v>
       </c>
@@ -867,7 +867,7 @@
         <v>55.616748804048804</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2022</v>
       </c>
@@ -892,9 +892,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{209B4BF9-A1A2-42A3-B429-B839E2C11906}">
   <dimension ref="A1:F27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -914,7 +914,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2021</v>
       </c>
@@ -931,7 +931,7 @@
         <v>0.116534014851655</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2021</v>
       </c>
@@ -948,7 +948,7 @@
         <v>0.102866612966851</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2021</v>
       </c>
@@ -965,7 +965,7 @@
         <v>0.20435531964029599</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -982,7 +982,7 @@
         <v>0.25130632032893901</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2021</v>
       </c>
@@ -999,7 +999,7 @@
         <v>0.276744983034311</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2021</v>
       </c>
@@ -1016,7 +1016,7 @@
         <v>0.27874363365664001</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2021</v>
       </c>
@@ -1033,7 +1033,7 @@
         <v>0.34345523368708603</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2021</v>
       </c>
@@ -1050,7 +1050,7 @@
         <v>0.54373684192649896</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2021</v>
       </c>
@@ -1067,7 +1067,7 @@
         <v>0.66955986420790603</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2021</v>
       </c>
@@ -1084,7 +1084,7 @@
         <v>0.61715456944164404</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2021</v>
       </c>
@@ -1101,7 +1101,7 @@
         <v>0.966130676412568</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2021</v>
       </c>
@@ -1118,7 +1118,7 @@
         <v>1.0318237124068199</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2021</v>
       </c>
@@ -1135,7 +1135,7 @@
         <v>0.97899999999999998</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2022</v>
       </c>
@@ -1152,7 +1152,7 @@
         <v>5.5776879862488103E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2022</v>
       </c>
@@ -1169,7 +1169,7 @@
         <v>0.13239207352472501</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2022</v>
       </c>
@@ -1186,7 +1186,7 @@
         <v>0.13480886246734899</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2022</v>
       </c>
@@ -1203,7 +1203,7 @@
         <v>0.22316621871325801</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2022</v>
       </c>
@@ -1220,7 +1220,7 @@
         <v>0.31089919407556099</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2022</v>
       </c>
@@ -1237,7 +1237,7 @@
         <v>0.42430924962455702</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2022</v>
       </c>
@@ -1254,7 +1254,7 @@
         <v>0.55437167658233699</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2022</v>
       </c>
@@ -1271,7 +1271,7 @@
         <v>0.68186126534474101</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2022</v>
       </c>
@@ -1288,7 +1288,7 @@
         <v>0.82442507725390901</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2022</v>
       </c>
@@ -1305,7 +1305,7 @@
         <v>1.01115180316078</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2022</v>
       </c>
@@ -1322,7 +1322,7 @@
         <v>1.1531750825354801</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2022</v>
       </c>
@@ -1339,7 +1339,7 @@
         <v>1.27014485187954</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2022</v>
       </c>
@@ -1364,9 +1364,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{045D14A7-CC75-44C0-8FF4-8DE7C82A1AA5}">
   <dimension ref="A1:F201"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1386,7 +1386,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2021</v>
       </c>
@@ -1397,7 +1397,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2021</v>
       </c>
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2021</v>
       </c>
@@ -1419,7 +1419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -1430,7 +1430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2021</v>
       </c>
@@ -1441,7 +1441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2021</v>
       </c>
@@ -1452,7 +1452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2021</v>
       </c>
@@ -1463,7 +1463,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2021</v>
       </c>
@@ -1474,7 +1474,7 @@
         <v>2.8201799306749868</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2021</v>
       </c>
@@ -1485,7 +1485,7 @@
         <v>64.554762462298399</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2021</v>
       </c>
@@ -1496,7 +1496,7 @@
         <v>183.6265003573065</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2021</v>
       </c>
@@ -1507,7 +1507,7 @@
         <v>302.11210216096998</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2021</v>
       </c>
@@ -1518,7 +1518,7 @@
         <v>559.29815066509991</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2021</v>
       </c>
@@ -1529,7 +1529,7 @@
         <v>574.1431641314</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2021</v>
       </c>
@@ -1540,7 +1540,7 @@
         <v>504.09790965470006</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2021</v>
       </c>
@@ -1551,7 +1551,7 @@
         <v>186.56927303576009</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2021</v>
       </c>
@@ -1562,7 +1562,7 @@
         <v>12.20623271879011</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2021</v>
       </c>
@@ -1573,7 +1573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2021</v>
       </c>
@@ -1584,7 +1584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2021</v>
       </c>
@@ -1595,7 +1595,7 @@
         <v>5.3231057104999903E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2021</v>
       </c>
@@ -1606,7 +1606,7 @@
         <v>2.1789700402895003</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2021</v>
       </c>
@@ -1617,7 +1617,7 @@
         <v>9.6756136043474861</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2021</v>
       </c>
@@ -1628,7 +1628,7 @@
         <v>33.835117365456369</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2021</v>
       </c>
@@ -1639,7 +1639,7 @@
         <v>63.512867885973499</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2021</v>
       </c>
@@ -1650,7 +1650,7 @@
         <v>69.294219092570501</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2021</v>
       </c>
@@ -1661,7 +1661,7 @@
         <v>71.090608340238006</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2021</v>
       </c>
@@ -1672,7 +1672,7 @@
         <v>90.163484136774002</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2021</v>
       </c>
@@ -1683,7 +1683,7 @@
         <v>181.26799911174899</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>2021</v>
       </c>
@@ -1694,7 +1694,7 @@
         <v>341.54778234956177</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2021</v>
       </c>
@@ -1705,7 +1705,7 @@
         <v>549.23699179601533</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2021</v>
       </c>
@@ -1716,7 +1716,7 @@
         <v>1070.0059819357846</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2021</v>
       </c>
@@ -1727,7 +1727,7 @@
         <v>1707.547601797577</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2021</v>
       </c>
@@ -1738,7 +1738,7 @@
         <v>2433.5829613892606</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2021</v>
       </c>
@@ -1749,7 +1749,7 @@
         <v>4892.0138732744472</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>2021</v>
       </c>
@@ -1760,7 +1760,7 @@
         <v>8087.1903693842132</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>2021</v>
       </c>
@@ -1771,7 +1771,7 @@
         <v>10393.057877159206</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>2021</v>
       </c>
@@ -1782,7 +1782,7 @@
         <v>13831.510575354607</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>2021</v>
       </c>
@@ -1793,7 +1793,7 @@
         <v>16428.837527138443</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2021</v>
       </c>
@@ -1804,7 +1804,7 @@
         <v>16081.033977088751</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>2021</v>
       </c>
@@ -1815,7 +1815,7 @@
         <v>20231.450770365704</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>2021</v>
       </c>
@@ -1826,7 +1826,7 @@
         <v>19205.259508077092</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>2021</v>
       </c>
@@ -1837,7 +1837,7 @@
         <v>18998.419122843039</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>2021</v>
       </c>
@@ -1848,7 +1848,7 @@
         <v>13489.728098068908</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>2021</v>
       </c>
@@ -1859,7 +1859,7 @@
         <v>9626.7375855313148</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>2021</v>
       </c>
@@ -1870,7 +1870,7 @@
         <v>5685.150680028707</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>2021</v>
       </c>
@@ -1881,7 +1881,7 @@
         <v>3353.0061332444147</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>2021</v>
       </c>
@@ -1892,7 +1892,7 @@
         <v>2008.7792898125549</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2021</v>
       </c>
@@ -1903,7 +1903,7 @@
         <v>954.96511146024795</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>2021</v>
       </c>
@@ -1914,7 +1914,7 @@
         <v>396.37045205269931</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>2021</v>
       </c>
@@ -1925,7 +1925,7 @@
         <v>190.76478464681657</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>2021</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>115.77275663523649</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>2021</v>
       </c>
@@ -1947,7 +1947,7 @@
         <v>54.800240989962113</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>2021</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>28.234603685526</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>2021</v>
       </c>
@@ -1969,7 +1969,7 @@
         <v>17.954809290884999</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>2021</v>
       </c>
@@ -1980,7 +1980,7 @@
         <v>11.680994615029499</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>2021</v>
       </c>
@@ -1991,7 +1991,7 @@
         <v>5.1148877436809999</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>2021</v>
       </c>
@@ -2002,7 +2002,7 @@
         <v>2.7690687188099901</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>2021</v>
       </c>
@@ -2013,7 +2013,7 @@
         <v>0.48360273742950199</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>2021</v>
       </c>
@@ -2024,7 +2024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>2021</v>
       </c>
@@ -2035,7 +2035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>2021</v>
       </c>
@@ -2046,7 +2046,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>2021</v>
       </c>
@@ -2057,7 +2057,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>2021</v>
       </c>
@@ -2068,7 +2068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>2021</v>
       </c>
@@ -2079,7 +2079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>2021</v>
       </c>
@@ -2090,7 +2090,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>2021</v>
       </c>
@@ -2101,7 +2101,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>2021</v>
       </c>
@@ -2112,7 +2112,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>2021</v>
       </c>
@@ -2123,7 +2123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>2021</v>
       </c>
@@ -2134,7 +2134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>2021</v>
       </c>
@@ -2145,7 +2145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>2021</v>
       </c>
@@ -2156,7 +2156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>2021</v>
       </c>
@@ -2167,7 +2167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>2021</v>
       </c>
@@ -2178,7 +2178,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>2021</v>
       </c>
@@ -2189,7 +2189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>2021</v>
       </c>
@@ -2200,7 +2200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>2021</v>
       </c>
@@ -2211,7 +2211,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>2021</v>
       </c>
@@ -2222,7 +2222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>2021</v>
       </c>
@@ -2233,7 +2233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>2021</v>
       </c>
@@ -2244,7 +2244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>2021</v>
       </c>
@@ -2255,7 +2255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>2021</v>
       </c>
@@ -2266,7 +2266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>2021</v>
       </c>
@@ -2277,7 +2277,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>2021</v>
       </c>
@@ -2288,7 +2288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>2021</v>
       </c>
@@ -2299,7 +2299,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>2021</v>
       </c>
@@ -2310,7 +2310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>2021</v>
       </c>
@@ -2321,7 +2321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>2021</v>
       </c>
@@ -2332,7 +2332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>2021</v>
       </c>
@@ -2343,7 +2343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>2021</v>
       </c>
@@ -2354,7 +2354,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>2021</v>
       </c>
@@ -2365,7 +2365,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>2021</v>
       </c>
@@ -2376,7 +2376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>2021</v>
       </c>
@@ -2387,7 +2387,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>2021</v>
       </c>
@@ -2398,7 +2398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>2021</v>
       </c>
@@ -2409,7 +2409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>2021</v>
       </c>
@@ -2420,7 +2420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>2021</v>
       </c>
@@ -2431,7 +2431,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>2021</v>
       </c>
@@ -2442,7 +2442,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>2021</v>
       </c>
@@ -2453,7 +2453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>2021</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>2021</v>
       </c>
@@ -2475,7 +2475,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>2021</v>
       </c>
@@ -2486,7 +2486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>2022</v>
       </c>
@@ -2497,7 +2497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>2022</v>
       </c>
@@ -2508,7 +2508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>2022</v>
       </c>
@@ -2519,7 +2519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>2022</v>
       </c>
@@ -2530,7 +2530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>2022</v>
       </c>
@@ -2541,7 +2541,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>2022</v>
       </c>
@@ -2552,7 +2552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>2022</v>
       </c>
@@ -2563,7 +2563,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>2022</v>
       </c>
@@ -2574,7 +2574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>2022</v>
       </c>
@@ -2585,7 +2585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>2022</v>
       </c>
@@ -2596,7 +2596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>2022</v>
       </c>
@@ -2607,7 +2607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>2022</v>
       </c>
@@ -2618,7 +2618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>2022</v>
       </c>
@@ -2629,7 +2629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>2022</v>
       </c>
@@ -2640,7 +2640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>2022</v>
       </c>
@@ -2651,7 +2651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>2022</v>
       </c>
@@ -2662,7 +2662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>2022</v>
       </c>
@@ -2673,7 +2673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>2022</v>
       </c>
@@ -2684,7 +2684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>2022</v>
       </c>
@@ -2695,7 +2695,7 @@
         <v>7.1609623311499879E-2</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>2022</v>
       </c>
@@ -2706,7 +2706,7 @@
         <v>0.1766039756885</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>2022</v>
       </c>
@@ -2717,7 +2717,7 @@
         <v>0.123081759254</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>2022</v>
       </c>
@@ -2728,7 +2728,7 @@
         <v>0.29291840883149989</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>2022</v>
       </c>
@@ -2739,7 +2739,7 @@
         <v>1.127187412339498</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>2022</v>
       </c>
@@ -2750,7 +2750,7 @@
         <v>15.827774774465</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>2022</v>
       </c>
@@ -2761,7 +2761,7 @@
         <v>331.93595320218401</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>2022</v>
       </c>
@@ -2772,7 +2772,7 @@
         <v>90.082071603572814</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>2022</v>
       </c>
@@ -2783,7 +2783,7 @@
         <v>96.780068814085496</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>2022</v>
       </c>
@@ -2794,7 +2794,7 @@
         <v>137.74040325472225</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>2022</v>
       </c>
@@ -2805,7 +2805,7 @@
         <v>276.52483305577289</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>2022</v>
       </c>
@@ -2816,7 +2816,7 @@
         <v>553.31027439822424</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>2022</v>
       </c>
@@ -2827,7 +2827,7 @@
         <v>1623.0014187674067</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>2022</v>
       </c>
@@ -2838,7 +2838,7 @@
         <v>3244.1507701096702</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>2022</v>
       </c>
@@ -2849,7 +2849,7 @@
         <v>4621.4534245142313</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>2022</v>
       </c>
@@ -2860,7 +2860,7 @@
         <v>6869.5734843701803</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>2022</v>
       </c>
@@ -2871,7 +2871,7 @@
         <v>9343.5694980515236</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>2022</v>
       </c>
@@ -2882,7 +2882,7 @@
         <v>10741.249014918068</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>2022</v>
       </c>
@@ -2893,7 +2893,7 @@
         <v>11460.938310951942</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>2022</v>
       </c>
@@ -2904,7 +2904,7 @@
         <v>11371.404409330289</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>2022</v>
       </c>
@@ -2915,7 +2915,7 @@
         <v>8857.7038375369375</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>2022</v>
       </c>
@@ -2926,7 +2926,7 @@
         <v>10578.992903711884</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>2022</v>
       </c>
@@ -2937,7 +2937,7 @@
         <v>12650.057365615889</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>2022</v>
       </c>
@@ -2948,7 +2948,7 @@
         <v>12211.458500861516</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>2022</v>
       </c>
@@ -2959,7 +2959,7 @@
         <v>12863.951377134512</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>2022</v>
       </c>
@@ -2970,7 +2970,7 @@
         <v>12058.760144656309</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>2022</v>
       </c>
@@ -2981,7 +2981,7 @@
         <v>9521.3892507828004</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>2022</v>
       </c>
@@ -2992,7 +2992,7 @@
         <v>6082.3238145867126</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>2022</v>
       </c>
@@ -3003,7 +3003,7 @@
         <v>3065.4458996021872</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>2022</v>
       </c>
@@ -3014,7 +3014,7 @@
         <v>2405.1753673126555</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>2022</v>
       </c>
@@ -3025,7 +3025,7 @@
         <v>1280.45909871711</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>2022</v>
       </c>
@@ -3036,7 +3036,7 @@
         <v>914.58144014917366</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>2022</v>
       </c>
@@ -3047,7 +3047,7 @@
         <v>548.51957858006165</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>2022</v>
       </c>
@@ -3058,7 +3058,7 @@
         <v>301.72147175036741</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>2022</v>
       </c>
@@ -3069,7 +3069,7 @@
         <v>90.525027492290107</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>2022</v>
       </c>
@@ -3080,7 +3080,7 @@
         <v>51.313238342125494</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>2022</v>
       </c>
@@ -3091,7 +3091,7 @@
         <v>62.476143627928515</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>2022</v>
       </c>
@@ -3102,7 +3102,7 @@
         <v>67.083169473299776</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>2022</v>
       </c>
@@ -3113,7 +3113,7 @@
         <v>37.015179186828128</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>2022</v>
       </c>
@@ -3124,7 +3124,7 @@
         <v>25.8192847209055</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>2022</v>
       </c>
@@ -3135,7 +3135,7 @@
         <v>12.966789139382501</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>2022</v>
       </c>
@@ -3146,7 +3146,7 @@
         <v>13.824365552383</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>2022</v>
       </c>
@@ -3157,7 +3157,7 @@
         <v>5.3752360985020102</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>2022</v>
       </c>
@@ -3168,7 +3168,7 @@
         <v>6.3512373028450098</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>2022</v>
       </c>
@@ -3179,7 +3179,7 @@
         <v>2.2106421196375199</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>2022</v>
       </c>
@@ -3190,7 +3190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>2022</v>
       </c>
@@ -3201,7 +3201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>2022</v>
       </c>
@@ -3212,7 +3212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>2022</v>
       </c>
@@ -3223,7 +3223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>2022</v>
       </c>
@@ -3234,7 +3234,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>2022</v>
       </c>
@@ -3245,7 +3245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>2022</v>
       </c>
@@ -3256,7 +3256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>2022</v>
       </c>
@@ -3267,7 +3267,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>2022</v>
       </c>
@@ -3278,7 +3278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>2022</v>
       </c>
@@ -3289,7 +3289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>2022</v>
       </c>
@@ -3300,7 +3300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>2022</v>
       </c>
@@ -3311,7 +3311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>2022</v>
       </c>
@@ -3322,7 +3322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>2022</v>
       </c>
@@ -3333,7 +3333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>2022</v>
       </c>
@@ -3344,7 +3344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>2022</v>
       </c>
@@ -3355,7 +3355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>2022</v>
       </c>
@@ -3366,7 +3366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>2022</v>
       </c>
@@ -3377,7 +3377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>2022</v>
       </c>
@@ -3388,7 +3388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>2022</v>
       </c>
@@ -3399,7 +3399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>2022</v>
       </c>
@@ -3410,7 +3410,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>2022</v>
       </c>
@@ -3421,7 +3421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>2022</v>
       </c>
@@ -3432,7 +3432,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>2022</v>
       </c>
@@ -3443,7 +3443,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>2022</v>
       </c>
@@ -3454,7 +3454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>2022</v>
       </c>
@@ -3465,7 +3465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>2022</v>
       </c>
@@ -3476,7 +3476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>2022</v>
       </c>
@@ -3487,7 +3487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>2022</v>
       </c>
@@ -3498,7 +3498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>2022</v>
       </c>
@@ -3509,7 +3509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>2022</v>
       </c>
@@ -3520,7 +3520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>2022</v>
       </c>
@@ -3531,7 +3531,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197">
         <v>2022</v>
       </c>
@@ -3542,7 +3542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198">
         <v>2022</v>
       </c>
@@ -3553,7 +3553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199">
         <v>2022</v>
       </c>
@@ -3564,7 +3564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200">
         <v>2022</v>
       </c>
@@ -3575,7 +3575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201">
         <v>2022</v>
       </c>
@@ -3594,9 +3594,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7886E624-8038-4FB5-9240-586936FC87C7}">
   <dimension ref="A1:E54"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3613,72 +3613,72 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1970</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1971</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1972</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1973</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1974</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1975</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1976</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1977</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1978</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>1979</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>1980</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1981</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>1982</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>1983</v>
       </c>
@@ -3686,7 +3686,7 @@
         <v>0.83735912891840636</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>1984</v>
       </c>
@@ -3694,7 +3694,7 @@
         <v>0.77011463323188944</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>1985</v>
       </c>
@@ -3702,7 +3702,7 @@
         <v>0.67320229191258063</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>1986</v>
       </c>
@@ -3710,7 +3710,7 @@
         <v>0.56654696253703873</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>1987</v>
       </c>
@@ -3718,7 +3718,7 @@
         <v>0.66592278567748997</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>1988</v>
       </c>
@@ -3726,7 +3726,7 @@
         <v>0.58482817820161326</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>1989</v>
       </c>
@@ -3734,7 +3734,7 @@
         <v>0.56915424702841144</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>1990</v>
       </c>
@@ -3742,7 +3742,7 @@
         <v>0.48727498047163748</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>1991</v>
       </c>
@@ -3750,7 +3750,7 @@
         <v>0.53717566399322125</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>1992</v>
       </c>
@@ -3758,7 +3758,7 @@
         <v>0.49184026401692127</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>1993</v>
       </c>
@@ -3766,7 +3766,7 @@
         <v>0.44059322955914987</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>1994</v>
       </c>
@@ -3774,7 +3774,7 @@
         <v>0.4734553178106175</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>1995</v>
       </c>
@@ -3782,7 +3782,7 @@
         <v>0.42284820237004195</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>1996</v>
       </c>
@@ -3790,7 +3790,7 @@
         <v>0.41801452833324715</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>1997</v>
       </c>
@@ -3798,7 +3798,7 @@
         <v>0.3427163026187699</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>1998</v>
       </c>
@@ -3806,7 +3806,7 @@
         <v>0.29086868916856573</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>1999</v>
       </c>
@@ -3814,7 +3814,7 @@
         <v>0.2962660005419242</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2000</v>
       </c>
@@ -3822,7 +3822,7 @@
         <v>0.2862018250229692</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2001</v>
       </c>
@@ -3830,7 +3830,7 @@
         <v>0.34118423312516732</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2002</v>
       </c>
@@ -3841,7 +3841,7 @@
         <v>4.0654954238624903</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>2003</v>
       </c>
@@ -3849,10 +3849,10 @@
         <v>0.26018365671645394</v>
       </c>
       <c r="D35">
-        <v>4.8017060784259797</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+        <v>4.7536890176417197</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>2004</v>
       </c>
@@ -3860,10 +3860,10 @@
         <v>0.28114393345652267</v>
       </c>
       <c r="D36">
-        <v>5.2893101103582003</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+        <v>5.1840528391620717</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>2005</v>
       </c>
@@ -3871,10 +3871,10 @@
         <v>0.25502971340298169</v>
       </c>
       <c r="D37">
-        <v>4.1933216761063496</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+        <v>4.0687758290043146</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>2006</v>
       </c>
@@ -3882,10 +3882,10 @@
         <v>0.2764783617192848</v>
       </c>
       <c r="D38">
-        <v>5.5767758409228403</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+        <v>5.3570286214548748</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2007</v>
       </c>
@@ -3893,10 +3893,10 @@
         <v>0.207045067437443</v>
       </c>
       <c r="D39">
-        <v>7.8127451575115501</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+        <v>7.4298429071978918</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>2008</v>
       </c>
@@ -3904,13 +3904,13 @@
         <v>0.13602629951072664</v>
       </c>
       <c r="D40">
-        <v>4.0045901917550104</v>
+        <v>3.7702421720232859</v>
       </c>
       <c r="E40">
         <v>1683.81871747838</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>2009</v>
       </c>
@@ -3918,13 +3918,13 @@
         <v>0.11288140570772709</v>
       </c>
       <c r="D41">
-        <v>1.4352765636122</v>
+        <v>1.3377715496059541</v>
       </c>
       <c r="E41">
         <v>1171.55141113847</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>2010</v>
       </c>
@@ -3932,13 +3932,13 @@
         <v>8.6825813818750944E-2</v>
       </c>
       <c r="D42">
-        <v>2.6957076603172299</v>
+        <v>2.4874499412864255</v>
       </c>
       <c r="E42">
         <v>823.90903816108096</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>2011</v>
       </c>
@@ -3946,13 +3946,13 @@
         <v>4.8078014640744487E-2</v>
       </c>
       <c r="D43">
-        <v>6.9229286160998296</v>
+        <v>6.3242146939052466</v>
       </c>
       <c r="E43">
         <v>733.50314991437801</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>2012</v>
       </c>
@@ -3960,13 +3960,13 @@
         <v>0.14692886845355663</v>
       </c>
       <c r="D44">
-        <v>6.1037758006070701</v>
+        <v>5.5201454239415479</v>
       </c>
       <c r="E44">
         <v>622.27342293794595</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>2013</v>
       </c>
@@ -3974,13 +3974,13 @@
         <v>0.1287745254844371</v>
       </c>
       <c r="D45">
-        <v>2.7246691992394201</v>
+        <v>2.4395005642795167</v>
       </c>
       <c r="E45">
         <v>707.99382958407602</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>2014</v>
       </c>
@@ -3988,13 +3988,13 @@
         <v>0.10159765722830148</v>
       </c>
       <c r="D46">
-        <v>3.7433119984161101</v>
+        <v>3.3180151255095107</v>
       </c>
       <c r="E46">
         <v>741.39002083147102</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>2015</v>
       </c>
@@ -4002,13 +4002,13 @@
         <v>8.3421541460967377E-2</v>
       </c>
       <c r="D47">
-        <v>3.0184971334804001</v>
+        <v>2.6487946924911725</v>
       </c>
       <c r="E47">
         <v>1009.29260487027</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2016</v>
       </c>
@@ -4016,13 +4016,13 @@
         <v>0.14983739649902303</v>
       </c>
       <c r="D48">
-        <v>2.6203602468230001</v>
+        <v>2.2764269923737674</v>
       </c>
       <c r="E48">
         <v>728.14759760899699</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>2017</v>
       </c>
@@ -4030,13 +4030,13 @@
         <v>0.17848137316231133</v>
       </c>
       <c r="D49">
-        <v>3.3940643451237298</v>
+        <v>2.9190933962137766</v>
       </c>
       <c r="E49">
         <v>935.77803374597397</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>2018</v>
       </c>
@@ -4044,13 +4044,13 @@
         <v>0.17944404803261474</v>
       </c>
       <c r="D50">
-        <v>9.5949614473138407</v>
+        <v>8.1697044876711029</v>
       </c>
       <c r="E50">
         <v>800.29460316653103</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>2019</v>
       </c>
@@ -4058,13 +4058,13 @@
         <v>0.19723851360485473</v>
       </c>
       <c r="D51">
-        <v>16.256122490136701</v>
+        <v>13.7029878038761</v>
       </c>
       <c r="E51">
         <v>972.16130815182703</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>2020</v>
       </c>
@@ -4072,10 +4072,10 @@
         <v>0.25758585644585547</v>
       </c>
       <c r="D52">
-        <v>17.960443762385999</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+        <v>14.9882374814615</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>2021</v>
       </c>
@@ -4083,13 +4083,13 @@
         <v>0.27130858289013526</v>
       </c>
       <c r="D53">
-        <v>21.868564419848799</v>
+        <v>18.067121772006352</v>
       </c>
       <c r="E53">
         <v>1555.9097129622401</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>2022</v>
       </c>
@@ -4097,7 +4097,7 @@
         <v>0.32336403536054648</v>
       </c>
       <c r="D54">
-        <v>24.905782669698699</v>
+        <v>20.370612431835443</v>
       </c>
     </row>
   </sheetData>
@@ -4108,9 +4108,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E42CCE45-3DDC-4861-A006-F4C4C7145E6D}">
   <dimension ref="A1:G27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -4133,7 +4133,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2021</v>
       </c>
@@ -4144,7 +4144,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2021</v>
       </c>
@@ -4158,7 +4158,7 @@
         <v>7583889.6923095835</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2021</v>
       </c>
@@ -4172,7 +4172,7 @@
         <v>595227.3525690505</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -4189,7 +4189,7 @@
         <v>12326.4818</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2021</v>
       </c>
@@ -4206,7 +4206,7 @@
         <v>132128.80092257101</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2021</v>
       </c>
@@ -4223,7 +4223,7 @@
         <v>254900.440891734</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2021</v>
       </c>
@@ -4240,7 +4240,7 @@
         <v>309959.65336691099</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2021</v>
       </c>
@@ -4257,7 +4257,7 @@
         <v>303061.70799844101</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2021</v>
       </c>
@@ -4274,7 +4274,7 @@
         <v>204906.68145700899</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2021</v>
       </c>
@@ -4291,7 +4291,7 @@
         <v>54827.885250500003</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2021</v>
       </c>
@@ -4305,7 +4305,7 @@
         <v>40133.928883433298</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2021</v>
       </c>
@@ -4319,7 +4319,7 @@
         <v>1956.6304683000001</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2021</v>
       </c>
@@ -4333,9 +4333,9 @@
         <v>608.6725199</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -4344,9 +4344,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -4358,9 +4358,9 @@
         <v>3.0881634275280619E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B17">
         <v>2</v>
@@ -4372,9 +4372,9 @@
         <v>0.21873656086941168</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B18">
         <v>3</v>
@@ -4389,9 +4389,9 @@
         <v>0.39652557711957498</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B19">
         <v>4</v>
@@ -4406,9 +4406,9 @@
         <v>0.64835381225940203</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B20">
         <v>5</v>
@@ -4423,9 +4423,9 @@
         <v>0.66442774174667596</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B21">
         <v>6</v>
@@ -4440,9 +4440,9 @@
         <v>0.84281146013221098</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B22">
         <v>7</v>
@@ -4457,9 +4457,9 @@
         <v>0.91046321547934606</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B23">
         <v>8</v>
@@ -4474,9 +4474,9 @@
         <v>1.30937140418139</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B24">
         <v>9</v>
@@ -4491,9 +4491,9 @@
         <v>1.3559045186261001</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B25">
         <v>10</v>
@@ -4505,9 +4505,9 @@
         <v>1.64690578852612</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B26">
         <v>11</v>
@@ -4519,9 +4519,9 @@
         <v>2.62620886093926</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B27">
         <v>12</v>
@@ -4539,9 +4539,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4691,19 +4694,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2AFB9C7-A01A-423B-A442-B6889BA2E519}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{228CE105-4287-40ED-B72B-E33A77B67D61}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4727,9 +4726,10 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{228CE105-4287-40ED-B72B-E33A77B67D61}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2AFB9C7-A01A-423B-A442-B6889BA2E519}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
bug fix to input file
</commit_message>
<xml_diff>
--- a/assessment/data/SC10_2022assessmentInputData.xlsx
+++ b/assessment/data/SC10_2022assessmentInputData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://southpacificrfmo.sharepoint.com/sites/SPRFMOSCJackMackerelWorkingGroup/Shared Documents/Data repository/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leeqi/Desktop/SPRFMO/jjm/assessment/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2BB3040E-2287-40B5-ABC1-96FD71463E9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9B78803-B97F-E34C-9E06-1651F035236E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="840" yWindow="-120" windowWidth="28080" windowHeight="16440" activeTab="3" xr2:uid="{11C67D07-EBA6-4D97-A3E6-A5FACAECFD42}"/>
+    <workbookView xWindow="840" yWindow="500" windowWidth="28080" windowHeight="16440" activeTab="4" xr2:uid="{11C67D07-EBA6-4D97-A3E6-A5FACAECFD42}"/>
   </bookViews>
   <sheets>
     <sheet name="ageComps" sheetId="1" r:id="rId1"/>
@@ -423,9 +423,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCC02C38-8F7E-48D4-BE42-B6D35726D79C}">
   <dimension ref="A1:F27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -445,7 +445,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>2021</v>
       </c>
@@ -459,7 +459,7 @@
         <v>670.16183246731998</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2021</v>
       </c>
@@ -476,7 +476,7 @@
         <v>13279.648895886301</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2021</v>
       </c>
@@ -493,7 +493,7 @@
         <v>44760.811535680899</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -510,7 +510,7 @@
         <v>107827.383916946</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2021</v>
       </c>
@@ -527,7 +527,7 @@
         <v>28181.237063751298</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2021</v>
       </c>
@@ -544,7 +544,7 @@
         <v>15482.537721409301</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2021</v>
       </c>
@@ -561,7 +561,7 @@
         <v>4128.7939220620001</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2021</v>
       </c>
@@ -578,7 +578,7 @@
         <v>427.17024803910601</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2021</v>
       </c>
@@ -595,7 +595,7 @@
         <v>110.74670539676799</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2021</v>
       </c>
@@ -612,7 +612,7 @@
         <v>221.93965880599998</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2021</v>
       </c>
@@ -629,7 +629,7 @@
         <v>10.7458646434357</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2021</v>
       </c>
@@ -646,7 +646,7 @@
         <v>4.1277274962150202E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2021</v>
       </c>
@@ -663,7 +663,7 @@
         <v>3.48499840965275</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2022</v>
       </c>
@@ -680,7 +680,7 @@
         <v>566.99602958347407</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>2022</v>
       </c>
@@ -697,7 +697,7 @@
         <v>32809.856850873999</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>2022</v>
       </c>
@@ -714,7 +714,7 @@
         <v>178240.213244949</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>2022</v>
       </c>
@@ -731,7 +731,7 @@
         <v>7845.8419073151599</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>2022</v>
       </c>
@@ -748,7 +748,7 @@
         <v>3835.6966651638604</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>2022</v>
       </c>
@@ -765,7 +765,7 @@
         <v>2051.2549168066002</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>2022</v>
       </c>
@@ -782,7 +782,7 @@
         <v>929.75059235101901</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>2022</v>
       </c>
@@ -799,7 +799,7 @@
         <v>441.63141196245601</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>2022</v>
       </c>
@@ -816,7 +816,7 @@
         <v>263.18018713831498</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>2022</v>
       </c>
@@ -833,7 +833,7 @@
         <v>132.02478459123498</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>2022</v>
       </c>
@@ -850,7 +850,7 @@
         <v>78.603420554523197</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>2022</v>
       </c>
@@ -867,7 +867,7 @@
         <v>55.616748804048804</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>2022</v>
       </c>
@@ -892,9 +892,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{209B4BF9-A1A2-42A3-B429-B839E2C11906}">
   <dimension ref="A1:F27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -914,7 +914,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>2021</v>
       </c>
@@ -931,7 +931,7 @@
         <v>0.116534014851655</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2021</v>
       </c>
@@ -948,7 +948,7 @@
         <v>0.102866612966851</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2021</v>
       </c>
@@ -965,7 +965,7 @@
         <v>0.20435531964029599</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -982,7 +982,7 @@
         <v>0.25130632032893901</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2021</v>
       </c>
@@ -999,7 +999,7 @@
         <v>0.276744983034311</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2021</v>
       </c>
@@ -1016,7 +1016,7 @@
         <v>0.27874363365664001</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2021</v>
       </c>
@@ -1033,7 +1033,7 @@
         <v>0.34345523368708603</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2021</v>
       </c>
@@ -1050,7 +1050,7 @@
         <v>0.54373684192649896</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2021</v>
       </c>
@@ -1067,7 +1067,7 @@
         <v>0.66955986420790603</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2021</v>
       </c>
@@ -1084,7 +1084,7 @@
         <v>0.61715456944164404</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2021</v>
       </c>
@@ -1101,7 +1101,7 @@
         <v>0.966130676412568</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2021</v>
       </c>
@@ -1118,7 +1118,7 @@
         <v>1.0318237124068199</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2021</v>
       </c>
@@ -1135,7 +1135,7 @@
         <v>0.97899999999999998</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2022</v>
       </c>
@@ -1152,7 +1152,7 @@
         <v>5.5776879862488103E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>2022</v>
       </c>
@@ -1169,7 +1169,7 @@
         <v>0.13239207352472501</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>2022</v>
       </c>
@@ -1186,7 +1186,7 @@
         <v>0.13480886246734899</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>2022</v>
       </c>
@@ -1203,7 +1203,7 @@
         <v>0.22316621871325801</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>2022</v>
       </c>
@@ -1220,7 +1220,7 @@
         <v>0.31089919407556099</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>2022</v>
       </c>
@@ -1237,7 +1237,7 @@
         <v>0.42430924962455702</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>2022</v>
       </c>
@@ -1254,7 +1254,7 @@
         <v>0.55437167658233699</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>2022</v>
       </c>
@@ -1271,7 +1271,7 @@
         <v>0.68186126534474101</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>2022</v>
       </c>
@@ -1288,7 +1288,7 @@
         <v>0.82442507725390901</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>2022</v>
       </c>
@@ -1305,7 +1305,7 @@
         <v>1.01115180316078</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>2022</v>
       </c>
@@ -1322,7 +1322,7 @@
         <v>1.1531750825354801</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>2022</v>
       </c>
@@ -1339,7 +1339,7 @@
         <v>1.27014485187954</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>2022</v>
       </c>
@@ -1364,9 +1364,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{045D14A7-CC75-44C0-8FF4-8DE7C82A1AA5}">
   <dimension ref="A1:F201"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1386,7 +1386,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>2021</v>
       </c>
@@ -1397,7 +1397,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2021</v>
       </c>
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2021</v>
       </c>
@@ -1419,7 +1419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -1430,7 +1430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2021</v>
       </c>
@@ -1441,7 +1441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2021</v>
       </c>
@@ -1452,7 +1452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2021</v>
       </c>
@@ -1463,7 +1463,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2021</v>
       </c>
@@ -1474,7 +1474,7 @@
         <v>2.8201799306749868</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2021</v>
       </c>
@@ -1485,7 +1485,7 @@
         <v>64.554762462298399</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2021</v>
       </c>
@@ -1496,7 +1496,7 @@
         <v>183.6265003573065</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2021</v>
       </c>
@@ -1507,7 +1507,7 @@
         <v>302.11210216096998</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2021</v>
       </c>
@@ -1518,7 +1518,7 @@
         <v>559.29815066509991</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2021</v>
       </c>
@@ -1529,7 +1529,7 @@
         <v>574.1431641314</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2021</v>
       </c>
@@ -1540,7 +1540,7 @@
         <v>504.09790965470006</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>2021</v>
       </c>
@@ -1551,7 +1551,7 @@
         <v>186.56927303576009</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>2021</v>
       </c>
@@ -1562,7 +1562,7 @@
         <v>12.20623271879011</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>2021</v>
       </c>
@@ -1573,7 +1573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>2021</v>
       </c>
@@ -1584,7 +1584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>2021</v>
       </c>
@@ -1595,7 +1595,7 @@
         <v>5.3231057104999903E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>2021</v>
       </c>
@@ -1606,7 +1606,7 @@
         <v>2.1789700402895003</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>2021</v>
       </c>
@@ -1617,7 +1617,7 @@
         <v>9.6756136043474861</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>2021</v>
       </c>
@@ -1628,7 +1628,7 @@
         <v>33.835117365456369</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>2021</v>
       </c>
@@ -1639,7 +1639,7 @@
         <v>63.512867885973499</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>2021</v>
       </c>
@@ -1650,7 +1650,7 @@
         <v>69.294219092570501</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>2021</v>
       </c>
@@ -1661,7 +1661,7 @@
         <v>71.090608340238006</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>2021</v>
       </c>
@@ -1672,7 +1672,7 @@
         <v>90.163484136774002</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>2021</v>
       </c>
@@ -1683,7 +1683,7 @@
         <v>181.26799911174899</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>2021</v>
       </c>
@@ -1694,7 +1694,7 @@
         <v>341.54778234956177</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>2021</v>
       </c>
@@ -1705,7 +1705,7 @@
         <v>549.23699179601533</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>2021</v>
       </c>
@@ -1716,7 +1716,7 @@
         <v>1070.0059819357846</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>2021</v>
       </c>
@@ -1727,7 +1727,7 @@
         <v>1707.547601797577</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>2021</v>
       </c>
@@ -1738,7 +1738,7 @@
         <v>2433.5829613892606</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>2021</v>
       </c>
@@ -1749,7 +1749,7 @@
         <v>4892.0138732744472</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>2021</v>
       </c>
@@ -1760,7 +1760,7 @@
         <v>8087.1903693842132</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>2021</v>
       </c>
@@ -1771,7 +1771,7 @@
         <v>10393.057877159206</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>2021</v>
       </c>
@@ -1782,7 +1782,7 @@
         <v>13831.510575354607</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>2021</v>
       </c>
@@ -1793,7 +1793,7 @@
         <v>16428.837527138443</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>2021</v>
       </c>
@@ -1804,7 +1804,7 @@
         <v>16081.033977088751</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>2021</v>
       </c>
@@ -1815,7 +1815,7 @@
         <v>20231.450770365704</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>2021</v>
       </c>
@@ -1826,7 +1826,7 @@
         <v>19205.259508077092</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>2021</v>
       </c>
@@ -1837,7 +1837,7 @@
         <v>18998.419122843039</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>2021</v>
       </c>
@@ -1848,7 +1848,7 @@
         <v>13489.728098068908</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>2021</v>
       </c>
@@ -1859,7 +1859,7 @@
         <v>9626.7375855313148</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>2021</v>
       </c>
@@ -1870,7 +1870,7 @@
         <v>5685.150680028707</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>2021</v>
       </c>
@@ -1881,7 +1881,7 @@
         <v>3353.0061332444147</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>2021</v>
       </c>
@@ -1892,7 +1892,7 @@
         <v>2008.7792898125549</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>2021</v>
       </c>
@@ -1903,7 +1903,7 @@
         <v>954.96511146024795</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>2021</v>
       </c>
@@ -1914,7 +1914,7 @@
         <v>396.37045205269931</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>2021</v>
       </c>
@@ -1925,7 +1925,7 @@
         <v>190.76478464681657</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>2021</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>115.77275663523649</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>2021</v>
       </c>
@@ -1947,7 +1947,7 @@
         <v>54.800240989962113</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>2021</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>28.234603685526</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>2021</v>
       </c>
@@ -1969,7 +1969,7 @@
         <v>17.954809290884999</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>2021</v>
       </c>
@@ -1980,7 +1980,7 @@
         <v>11.680994615029499</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>2021</v>
       </c>
@@ -1991,7 +1991,7 @@
         <v>5.1148877436809999</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>2021</v>
       </c>
@@ -2002,7 +2002,7 @@
         <v>2.7690687188099901</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>2021</v>
       </c>
@@ -2013,7 +2013,7 @@
         <v>0.48360273742950199</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>2021</v>
       </c>
@@ -2024,7 +2024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>2021</v>
       </c>
@@ -2035,7 +2035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>2021</v>
       </c>
@@ -2046,7 +2046,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>2021</v>
       </c>
@@ -2057,7 +2057,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>2021</v>
       </c>
@@ -2068,7 +2068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>2021</v>
       </c>
@@ -2079,7 +2079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>2021</v>
       </c>
@@ -2090,7 +2090,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>2021</v>
       </c>
@@ -2101,7 +2101,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>2021</v>
       </c>
@@ -2112,7 +2112,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>2021</v>
       </c>
@@ -2123,7 +2123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>2021</v>
       </c>
@@ -2134,7 +2134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>2021</v>
       </c>
@@ -2145,7 +2145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>2021</v>
       </c>
@@ -2156,7 +2156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>2021</v>
       </c>
@@ -2167,7 +2167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>2021</v>
       </c>
@@ -2178,7 +2178,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>2021</v>
       </c>
@@ -2189,7 +2189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>2021</v>
       </c>
@@ -2200,7 +2200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>2021</v>
       </c>
@@ -2211,7 +2211,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>2021</v>
       </c>
@@ -2222,7 +2222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>2021</v>
       </c>
@@ -2233,7 +2233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>2021</v>
       </c>
@@ -2244,7 +2244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>2021</v>
       </c>
@@ -2255,7 +2255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>2021</v>
       </c>
@@ -2266,7 +2266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>2021</v>
       </c>
@@ -2277,7 +2277,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>2021</v>
       </c>
@@ -2288,7 +2288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>2021</v>
       </c>
@@ -2299,7 +2299,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>2021</v>
       </c>
@@ -2310,7 +2310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>2021</v>
       </c>
@@ -2321,7 +2321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>2021</v>
       </c>
@@ -2332,7 +2332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>2021</v>
       </c>
@@ -2343,7 +2343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>2021</v>
       </c>
@@ -2354,7 +2354,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>2021</v>
       </c>
@@ -2365,7 +2365,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>2021</v>
       </c>
@@ -2376,7 +2376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>2021</v>
       </c>
@@ -2387,7 +2387,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>2021</v>
       </c>
@@ -2398,7 +2398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>2021</v>
       </c>
@@ -2409,7 +2409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>2021</v>
       </c>
@@ -2420,7 +2420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>2021</v>
       </c>
@@ -2431,7 +2431,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>2021</v>
       </c>
@@ -2442,7 +2442,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>2021</v>
       </c>
@@ -2453,7 +2453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>2021</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>2021</v>
       </c>
@@ -2475,7 +2475,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>2021</v>
       </c>
@@ -2486,7 +2486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>2022</v>
       </c>
@@ -2497,7 +2497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>2022</v>
       </c>
@@ -2508,7 +2508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>2022</v>
       </c>
@@ -2519,7 +2519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>2022</v>
       </c>
@@ -2530,7 +2530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>2022</v>
       </c>
@@ -2541,7 +2541,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>2022</v>
       </c>
@@ -2552,7 +2552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>2022</v>
       </c>
@@ -2563,7 +2563,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>2022</v>
       </c>
@@ -2574,7 +2574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>2022</v>
       </c>
@@ -2585,7 +2585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>2022</v>
       </c>
@@ -2596,7 +2596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>2022</v>
       </c>
@@ -2607,7 +2607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A113">
         <v>2022</v>
       </c>
@@ -2618,7 +2618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A114">
         <v>2022</v>
       </c>
@@ -2629,7 +2629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A115">
         <v>2022</v>
       </c>
@@ -2640,7 +2640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A116">
         <v>2022</v>
       </c>
@@ -2651,7 +2651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A117">
         <v>2022</v>
       </c>
@@ -2662,7 +2662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A118">
         <v>2022</v>
       </c>
@@ -2673,7 +2673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A119">
         <v>2022</v>
       </c>
@@ -2684,7 +2684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A120">
         <v>2022</v>
       </c>
@@ -2695,7 +2695,7 @@
         <v>7.1609623311499879E-2</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A121">
         <v>2022</v>
       </c>
@@ -2706,7 +2706,7 @@
         <v>0.1766039756885</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A122">
         <v>2022</v>
       </c>
@@ -2717,7 +2717,7 @@
         <v>0.123081759254</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A123">
         <v>2022</v>
       </c>
@@ -2728,7 +2728,7 @@
         <v>0.29291840883149989</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A124">
         <v>2022</v>
       </c>
@@ -2739,7 +2739,7 @@
         <v>1.127187412339498</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A125">
         <v>2022</v>
       </c>
@@ -2750,7 +2750,7 @@
         <v>15.827774774465</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A126">
         <v>2022</v>
       </c>
@@ -2761,7 +2761,7 @@
         <v>331.93595320218401</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A127">
         <v>2022</v>
       </c>
@@ -2772,7 +2772,7 @@
         <v>90.082071603572814</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A128">
         <v>2022</v>
       </c>
@@ -2783,7 +2783,7 @@
         <v>96.780068814085496</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A129">
         <v>2022</v>
       </c>
@@ -2794,7 +2794,7 @@
         <v>137.74040325472225</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A130">
         <v>2022</v>
       </c>
@@ -2805,7 +2805,7 @@
         <v>276.52483305577289</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A131">
         <v>2022</v>
       </c>
@@ -2816,7 +2816,7 @@
         <v>553.31027439822424</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A132">
         <v>2022</v>
       </c>
@@ -2827,7 +2827,7 @@
         <v>1623.0014187674067</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A133">
         <v>2022</v>
       </c>
@@ -2838,7 +2838,7 @@
         <v>3244.1507701096702</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A134">
         <v>2022</v>
       </c>
@@ -2849,7 +2849,7 @@
         <v>4621.4534245142313</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A135">
         <v>2022</v>
       </c>
@@ -2860,7 +2860,7 @@
         <v>6869.5734843701803</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A136">
         <v>2022</v>
       </c>
@@ -2871,7 +2871,7 @@
         <v>9343.5694980515236</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A137">
         <v>2022</v>
       </c>
@@ -2882,7 +2882,7 @@
         <v>10741.249014918068</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A138">
         <v>2022</v>
       </c>
@@ -2893,7 +2893,7 @@
         <v>11460.938310951942</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A139">
         <v>2022</v>
       </c>
@@ -2904,7 +2904,7 @@
         <v>11371.404409330289</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A140">
         <v>2022</v>
       </c>
@@ -2915,7 +2915,7 @@
         <v>8857.7038375369375</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A141">
         <v>2022</v>
       </c>
@@ -2926,7 +2926,7 @@
         <v>10578.992903711884</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A142">
         <v>2022</v>
       </c>
@@ -2937,7 +2937,7 @@
         <v>12650.057365615889</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A143">
         <v>2022</v>
       </c>
@@ -2948,7 +2948,7 @@
         <v>12211.458500861516</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A144">
         <v>2022</v>
       </c>
@@ -2959,7 +2959,7 @@
         <v>12863.951377134512</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A145">
         <v>2022</v>
       </c>
@@ -2970,7 +2970,7 @@
         <v>12058.760144656309</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A146">
         <v>2022</v>
       </c>
@@ -2981,7 +2981,7 @@
         <v>9521.3892507828004</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A147">
         <v>2022</v>
       </c>
@@ -2992,7 +2992,7 @@
         <v>6082.3238145867126</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A148">
         <v>2022</v>
       </c>
@@ -3003,7 +3003,7 @@
         <v>3065.4458996021872</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A149">
         <v>2022</v>
       </c>
@@ -3014,7 +3014,7 @@
         <v>2405.1753673126555</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A150">
         <v>2022</v>
       </c>
@@ -3025,7 +3025,7 @@
         <v>1280.45909871711</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A151">
         <v>2022</v>
       </c>
@@ -3036,7 +3036,7 @@
         <v>914.58144014917366</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A152">
         <v>2022</v>
       </c>
@@ -3047,7 +3047,7 @@
         <v>548.51957858006165</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A153">
         <v>2022</v>
       </c>
@@ -3058,7 +3058,7 @@
         <v>301.72147175036741</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A154">
         <v>2022</v>
       </c>
@@ -3069,7 +3069,7 @@
         <v>90.525027492290107</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A155">
         <v>2022</v>
       </c>
@@ -3080,7 +3080,7 @@
         <v>51.313238342125494</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A156">
         <v>2022</v>
       </c>
@@ -3091,7 +3091,7 @@
         <v>62.476143627928515</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A157">
         <v>2022</v>
       </c>
@@ -3102,7 +3102,7 @@
         <v>67.083169473299776</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A158">
         <v>2022</v>
       </c>
@@ -3113,7 +3113,7 @@
         <v>37.015179186828128</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A159">
         <v>2022</v>
       </c>
@@ -3124,7 +3124,7 @@
         <v>25.8192847209055</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A160">
         <v>2022</v>
       </c>
@@ -3135,7 +3135,7 @@
         <v>12.966789139382501</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A161">
         <v>2022</v>
       </c>
@@ -3146,7 +3146,7 @@
         <v>13.824365552383</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A162">
         <v>2022</v>
       </c>
@@ -3157,7 +3157,7 @@
         <v>5.3752360985020102</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A163">
         <v>2022</v>
       </c>
@@ -3168,7 +3168,7 @@
         <v>6.3512373028450098</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A164">
         <v>2022</v>
       </c>
@@ -3179,7 +3179,7 @@
         <v>2.2106421196375199</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A165">
         <v>2022</v>
       </c>
@@ -3190,7 +3190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A166">
         <v>2022</v>
       </c>
@@ -3201,7 +3201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A167">
         <v>2022</v>
       </c>
@@ -3212,7 +3212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A168">
         <v>2022</v>
       </c>
@@ -3223,7 +3223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A169">
         <v>2022</v>
       </c>
@@ -3234,7 +3234,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A170">
         <v>2022</v>
       </c>
@@ -3245,7 +3245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A171">
         <v>2022</v>
       </c>
@@ -3256,7 +3256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A172">
         <v>2022</v>
       </c>
@@ -3267,7 +3267,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A173">
         <v>2022</v>
       </c>
@@ -3278,7 +3278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A174">
         <v>2022</v>
       </c>
@@ -3289,7 +3289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A175">
         <v>2022</v>
       </c>
@@ -3300,7 +3300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A176">
         <v>2022</v>
       </c>
@@ -3311,7 +3311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A177">
         <v>2022</v>
       </c>
@@ -3322,7 +3322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A178">
         <v>2022</v>
       </c>
@@ -3333,7 +3333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A179">
         <v>2022</v>
       </c>
@@ -3344,7 +3344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A180">
         <v>2022</v>
       </c>
@@ -3355,7 +3355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A181">
         <v>2022</v>
       </c>
@@ -3366,7 +3366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A182">
         <v>2022</v>
       </c>
@@ -3377,7 +3377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A183">
         <v>2022</v>
       </c>
@@ -3388,7 +3388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A184">
         <v>2022</v>
       </c>
@@ -3399,7 +3399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A185">
         <v>2022</v>
       </c>
@@ -3410,7 +3410,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A186">
         <v>2022</v>
       </c>
@@ -3421,7 +3421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A187">
         <v>2022</v>
       </c>
@@ -3432,7 +3432,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A188">
         <v>2022</v>
       </c>
@@ -3443,7 +3443,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A189">
         <v>2022</v>
       </c>
@@ -3454,7 +3454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A190">
         <v>2022</v>
       </c>
@@ -3465,7 +3465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A191">
         <v>2022</v>
       </c>
@@ -3476,7 +3476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A192">
         <v>2022</v>
       </c>
@@ -3487,7 +3487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A193">
         <v>2022</v>
       </c>
@@ -3498,7 +3498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A194">
         <v>2022</v>
       </c>
@@ -3509,7 +3509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A195">
         <v>2022</v>
       </c>
@@ -3520,7 +3520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A196">
         <v>2022</v>
       </c>
@@ -3531,7 +3531,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A197">
         <v>2022</v>
       </c>
@@ -3542,7 +3542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A198">
         <v>2022</v>
       </c>
@@ -3553,7 +3553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A199">
         <v>2022</v>
       </c>
@@ -3564,7 +3564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A200">
         <v>2022</v>
       </c>
@@ -3575,7 +3575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A201">
         <v>2022</v>
       </c>
@@ -3594,9 +3594,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7886E624-8038-4FB5-9240-586936FC87C7}">
   <dimension ref="A1:E54"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3613,72 +3613,72 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1970</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1971</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1972</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1973</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>1974</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>1975</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>1976</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>1977</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>1978</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>1979</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>1980</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>1981</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>1982</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>1983</v>
       </c>
@@ -3686,7 +3686,7 @@
         <v>0.83735912891840636</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>1984</v>
       </c>
@@ -3694,7 +3694,7 @@
         <v>0.77011463323188944</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>1985</v>
       </c>
@@ -3702,7 +3702,7 @@
         <v>0.67320229191258063</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>1986</v>
       </c>
@@ -3710,7 +3710,7 @@
         <v>0.56654696253703873</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>1987</v>
       </c>
@@ -3718,7 +3718,7 @@
         <v>0.66592278567748997</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>1988</v>
       </c>
@@ -3726,7 +3726,7 @@
         <v>0.58482817820161326</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>1989</v>
       </c>
@@ -3734,7 +3734,7 @@
         <v>0.56915424702841144</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>1990</v>
       </c>
@@ -3742,7 +3742,7 @@
         <v>0.48727498047163748</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>1991</v>
       </c>
@@ -3750,7 +3750,7 @@
         <v>0.53717566399322125</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>1992</v>
       </c>
@@ -3758,7 +3758,7 @@
         <v>0.49184026401692127</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>1993</v>
       </c>
@@ -3766,7 +3766,7 @@
         <v>0.44059322955914987</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>1994</v>
       </c>
@@ -3774,7 +3774,7 @@
         <v>0.4734553178106175</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>1995</v>
       </c>
@@ -3782,7 +3782,7 @@
         <v>0.42284820237004195</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>1996</v>
       </c>
@@ -3790,7 +3790,7 @@
         <v>0.41801452833324715</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>1997</v>
       </c>
@@ -3798,7 +3798,7 @@
         <v>0.3427163026187699</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>1998</v>
       </c>
@@ -3806,7 +3806,7 @@
         <v>0.29086868916856573</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>1999</v>
       </c>
@@ -3814,7 +3814,7 @@
         <v>0.2962660005419242</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>2000</v>
       </c>
@@ -3822,7 +3822,7 @@
         <v>0.2862018250229692</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>2001</v>
       </c>
@@ -3830,7 +3830,7 @@
         <v>0.34118423312516732</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>2002</v>
       </c>
@@ -3841,7 +3841,7 @@
         <v>4.0654954238624903</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>2003</v>
       </c>
@@ -3852,7 +3852,7 @@
         <v>4.7536890176417197</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>2004</v>
       </c>
@@ -3863,7 +3863,7 @@
         <v>5.1840528391620717</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>2005</v>
       </c>
@@ -3874,7 +3874,7 @@
         <v>4.0687758290043146</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>2006</v>
       </c>
@@ -3885,7 +3885,7 @@
         <v>5.3570286214548748</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>2007</v>
       </c>
@@ -3896,7 +3896,7 @@
         <v>7.4298429071978918</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>2008</v>
       </c>
@@ -3910,7 +3910,7 @@
         <v>1683.81871747838</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>2009</v>
       </c>
@@ -3924,7 +3924,7 @@
         <v>1171.55141113847</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>2010</v>
       </c>
@@ -3938,7 +3938,7 @@
         <v>823.90903816108096</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>2011</v>
       </c>
@@ -3952,7 +3952,7 @@
         <v>733.50314991437801</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>2012</v>
       </c>
@@ -3966,7 +3966,7 @@
         <v>622.27342293794595</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>2013</v>
       </c>
@@ -3980,7 +3980,7 @@
         <v>707.99382958407602</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>2014</v>
       </c>
@@ -3994,7 +3994,7 @@
         <v>741.39002083147102</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>2015</v>
       </c>
@@ -4008,7 +4008,7 @@
         <v>1009.29260487027</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>2016</v>
       </c>
@@ -4022,7 +4022,7 @@
         <v>728.14759760899699</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>2017</v>
       </c>
@@ -4036,7 +4036,7 @@
         <v>935.77803374597397</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>2018</v>
       </c>
@@ -4050,7 +4050,7 @@
         <v>800.29460316653103</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>2019</v>
       </c>
@@ -4064,7 +4064,7 @@
         <v>972.16130815182703</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>2020</v>
       </c>
@@ -4075,7 +4075,7 @@
         <v>14.9882374814615</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>2021</v>
       </c>
@@ -4089,7 +4089,7 @@
         <v>1555.9097129622401</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>2022</v>
       </c>
@@ -4108,9 +4108,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E42CCE45-3DDC-4861-A006-F4C4C7145E6D}">
   <dimension ref="A1:G27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -4133,7 +4133,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>2021</v>
       </c>
@@ -4144,7 +4144,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2021</v>
       </c>
@@ -4158,7 +4158,7 @@
         <v>7583889.6923095835</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2021</v>
       </c>
@@ -4172,7 +4172,7 @@
         <v>595227.3525690505</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -4189,7 +4189,7 @@
         <v>12326.4818</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2021</v>
       </c>
@@ -4206,7 +4206,7 @@
         <v>132128.80092257101</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2021</v>
       </c>
@@ -4223,7 +4223,7 @@
         <v>254900.440891734</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2021</v>
       </c>
@@ -4240,7 +4240,7 @@
         <v>309959.65336691099</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2021</v>
       </c>
@@ -4257,7 +4257,7 @@
         <v>303061.70799844101</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2021</v>
       </c>
@@ -4274,7 +4274,7 @@
         <v>204906.68145700899</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2021</v>
       </c>
@@ -4291,7 +4291,7 @@
         <v>54827.885250500003</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2021</v>
       </c>
@@ -4305,7 +4305,7 @@
         <v>40133.928883433298</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2021</v>
       </c>
@@ -4319,7 +4319,7 @@
         <v>1956.6304683000001</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2021</v>
       </c>
@@ -4333,9 +4333,9 @@
         <v>608.6725199</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -4344,9 +4344,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -4358,9 +4358,9 @@
         <v>3.0881634275280619E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B17">
         <v>2</v>
@@ -4372,9 +4372,9 @@
         <v>0.21873656086941168</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B18">
         <v>3</v>
@@ -4389,9 +4389,9 @@
         <v>0.39652557711957498</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B19">
         <v>4</v>
@@ -4406,9 +4406,9 @@
         <v>0.64835381225940203</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B20">
         <v>5</v>
@@ -4423,9 +4423,9 @@
         <v>0.66442774174667596</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B21">
         <v>6</v>
@@ -4440,9 +4440,9 @@
         <v>0.84281146013221098</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B22">
         <v>7</v>
@@ -4457,9 +4457,9 @@
         <v>0.91046321547934606</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B23">
         <v>8</v>
@@ -4474,9 +4474,9 @@
         <v>1.30937140418139</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B24">
         <v>9</v>
@@ -4491,9 +4491,9 @@
         <v>1.3559045186261001</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B25">
         <v>10</v>
@@ -4505,9 +4505,9 @@
         <v>1.64690578852612</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B26">
         <v>11</v>
@@ -4519,9 +4519,9 @@
         <v>2.62620886093926</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B27">
         <v>12</v>
@@ -4539,15 +4539,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100812D0B056278C642B7C89719D0EEC9C4" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="459ccd4a2f4db444801dd1c587af921d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f419981a-ca0a-4e56-9512-575f16b7ea2d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e76f6978cc275c7466d741305d3dbcb0" ns2:_="">
     <xsd:import namespace="f419981a-ca0a-4e56-9512-575f16b7ea2d"/>
@@ -4693,6 +4684,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -4700,14 +4700,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{228CE105-4287-40ED-B72B-E33A77B67D61}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85F76EC6-ADC5-49D9-8B88-F47A2495D4C8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4725,6 +4717,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{228CE105-4287-40ED-B72B-E33A77B67D61}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2AFB9C7-A01A-423B-A442-B6889BA2E519}">
   <ds:schemaRefs>

</xml_diff>